<commit_message>
feat: sincro diaria incremental, configuraciones de metas y mejoras visuales del front
</commit_message>
<xml_diff>
--- a/usuarios lista.xlsx
+++ b/usuarios lista.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="112">
   <si>
     <t>Usuario</t>
   </si>
@@ -330,6 +330,36 @@
   </si>
   <si>
     <t>nombre</t>
+  </si>
+  <si>
+    <t>Federico Pousa</t>
+  </si>
+  <si>
+    <t>fpousa</t>
+  </si>
+  <si>
+    <t>Fede2026</t>
+  </si>
+  <si>
+    <t>Paloma Malaspina</t>
+  </si>
+  <si>
+    <t>paloma</t>
+  </si>
+  <si>
+    <t>Palo2026</t>
+  </si>
+  <si>
+    <t>paloma.malaspina@gmail.com</t>
+  </si>
+  <si>
+    <t>ffedepousa@gmail.com</t>
+  </si>
+  <si>
+    <t>Federico Da Silva</t>
+  </si>
+  <si>
+    <t>fdasilva</t>
   </si>
 </sst>
 </file>
@@ -352,15 +382,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color theme="10"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -372,8 +402,13 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -381,20 +416,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Buena" xfId="1" builtinId="26"/>
-    <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
+    <cellStyle name="Celda de comprobación" xfId="2" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -673,7 +723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.5703125" customWidth="1"/>
@@ -684,449 +734,507 @@
     <col min="8" max="8" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:6" s="1" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E15" t="s">
-        <v>0</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="E15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="E16" t="s">
-        <v>0</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="E16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E17" t="s">
-        <v>0</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="E17" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E18" t="s">
-        <v>0</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="E18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E19" t="s">
-        <v>0</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="E19" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="E21" t="s">
-        <v>0</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="E21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E22" t="s">
-        <v>0</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="E22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1"/>
+    <hyperlink ref="F24" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>